<commit_message>
Tag archetype-specific columns in eval Excel headers (A1/A2, A2, B1)
</commit_message>
<xml_diff>
--- a/Prompt_Eval_Framework.xlsx
+++ b/Prompt_Eval_Framework.xlsx
@@ -616,14 +616,14 @@
     <col width="18" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
     <col width="18" customWidth="1" min="7" max="7"/>
-    <col width="16" customWidth="1" min="8" max="8"/>
-    <col width="14" customWidth="1" min="9" max="9"/>
-    <col width="18" customWidth="1" min="10" max="10"/>
-    <col width="14" customWidth="1" min="11" max="11"/>
-    <col width="14" customWidth="1" min="12" max="12"/>
-    <col width="14" customWidth="1" min="13" max="13"/>
+    <col width="20" customWidth="1" min="8" max="8"/>
+    <col width="18" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
+    <col width="18" customWidth="1" min="11" max="11"/>
+    <col width="16" customWidth="1" min="12" max="12"/>
+    <col width="16" customWidth="1" min="13" max="13"/>
     <col width="18" customWidth="1" min="14" max="14"/>
-    <col width="20" customWidth="1" min="15" max="15"/>
+    <col width="22" customWidth="1" min="15" max="15"/>
     <col width="16" customWidth="1" min="16" max="16"/>
     <col width="16" customWidth="1" min="17" max="17"/>
     <col width="14" customWidth="1" min="18" max="18"/>
@@ -708,47 +708,47 @@
       </c>
       <c r="H2" s="5" t="inlineStr">
         <is>
-          <t>Colour Palette</t>
+          <t>Colour Palette (A1/A2)</t>
         </is>
       </c>
       <c r="I2" s="5" t="inlineStr">
         <is>
-          <t>Bg Finish</t>
+          <t>Bg Finish (A1/A2)</t>
         </is>
       </c>
       <c r="J2" s="5" t="inlineStr">
         <is>
-          <t>Illustration</t>
+          <t>Illustration (A1/A2)</t>
         </is>
       </c>
       <c r="K2" s="5" t="inlineStr">
         <is>
-          <t>Render Style</t>
+          <t>Render Style (A1/A2)</t>
         </is>
       </c>
       <c r="L2" s="5" t="inlineStr">
         <is>
-          <t>Frame Deco</t>
+          <t>Frame Deco (A2)</t>
         </is>
       </c>
       <c r="M2" s="5" t="inlineStr">
         <is>
-          <t>Motif</t>
+          <t>Motif (A1/A2)</t>
         </is>
       </c>
       <c r="N2" s="5" t="inlineStr">
         <is>
-          <t>Scene Main</t>
+          <t>Scene Main (B1)</t>
         </is>
       </c>
       <c r="O2" s="5" t="inlineStr">
         <is>
-          <t>Scene Supporting</t>
+          <t>Scene Supporting (B1)</t>
         </is>
       </c>
       <c r="P2" s="5" t="inlineStr">
         <is>
-          <t>Mood</t>
+          <t>Mood (B1)</t>
         </is>
       </c>
       <c r="Q2" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Remove font/text from AI prompts - user adds text manually in post
- Remove font name refs from all 6 prompt builders
- Keep text overlay zone layout descriptions intact
- Strengthen no-text negatives across all platforms
- Add v18 docx with 61-entry clickable document index
- Update eval Excel with 4-platform columns and QA Testing Guide
- Char limits verified: Firefly max 951, Leonardo max 1326

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Prompt_Eval_Framework.xlsx
+++ b/Prompt_Eval_Framework.xlsx
@@ -10,6 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Eval Data" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Testing Guide" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -19,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="12">
+  <fonts count="17">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -90,8 +91,36 @@
       <color rgb="001E3A5F"/>
       <sz val="11"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="002563EB"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="0064748B"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <i val="1"/>
+      <color rgb="0064748B"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="001E3A5F"/>
+      <sz val="9"/>
+    </font>
   </fonts>
-  <fills count="14">
+  <fills count="21">
     <fill>
       <patternFill/>
     </fill>
@@ -158,6 +187,41 @@
         <fgColor rgb="00EFF6FF"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00B45309"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FEF2F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0078716C"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00475569"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00DB2777"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="000891B2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FEF3C7"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -185,7 +249,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="47">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -227,7 +291,7 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
+      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -240,6 +304,74 @@
     <xf numFmtId="0" fontId="11" fillId="13" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="14" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="16" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="15" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="15" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="15" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="15" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="16" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="18" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="19" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="13" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="20" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="20" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="20" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="20" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -606,7 +738,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AF11"/>
+  <dimension ref="A1:AG11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -631,16 +763,17 @@
     <col width="30" customWidth="1" min="20" max="20"/>
     <col width="30" customWidth="1" min="21" max="21"/>
     <col width="30" customWidth="1" min="22" max="22"/>
-    <col width="20" customWidth="1" min="23" max="23"/>
-    <col width="22" customWidth="1" min="24" max="24"/>
-    <col width="28" customWidth="1" min="25" max="25"/>
-    <col width="20" customWidth="1" min="26" max="26"/>
-    <col width="22" customWidth="1" min="27" max="27"/>
-    <col width="18" customWidth="1" min="28" max="28"/>
-    <col width="20" customWidth="1" min="29" max="29"/>
-    <col width="16" customWidth="1" min="30" max="30"/>
-    <col width="30" customWidth="1" min="31" max="31"/>
-    <col width="40" customWidth="1" min="32" max="32"/>
+    <col width="30" customWidth="1" min="23" max="23"/>
+    <col width="20" customWidth="1" min="24" max="24"/>
+    <col width="22" customWidth="1" min="25" max="25"/>
+    <col width="28" customWidth="1" min="26" max="26"/>
+    <col width="20" customWidth="1" min="27" max="27"/>
+    <col width="22" customWidth="1" min="28" max="28"/>
+    <col width="18" customWidth="1" min="29" max="29"/>
+    <col width="20" customWidth="1" min="30" max="30"/>
+    <col width="16" customWidth="1" min="31" max="31"/>
+    <col width="30" customWidth="1" min="32" max="32"/>
+    <col width="40" customWidth="1" min="33" max="33"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -649,22 +782,22 @@
           <t>PART A — Auto-Filled (Paste from Wizard Export)</t>
         </is>
       </c>
-      <c r="W1" s="2" t="inlineStr">
+      <c r="X1" s="2" t="inlineStr">
         <is>
           <t>① SCORE</t>
         </is>
       </c>
-      <c r="X1" s="2" t="inlineStr">
+      <c r="Y1" s="2" t="inlineStr">
         <is>
           <t>② ELEMENT CHECKS</t>
         </is>
       </c>
-      <c r="AC1" s="3" t="inlineStr">
+      <c r="AD1" s="3" t="inlineStr">
         <is>
           <t>③ LOOKS</t>
         </is>
       </c>
-      <c r="AF1" s="4" t="inlineStr">
+      <c r="AG1" s="4" t="inlineStr">
         <is>
           <t>④ NOTES</t>
         </is>
@@ -781,52 +914,57 @@
           <t>Prompt (Firefly)</t>
         </is>
       </c>
-      <c r="W2" s="6" t="inlineStr">
+      <c r="W2" s="5" t="inlineStr">
+        <is>
+          <t>Prompt (Gemini)</t>
+        </is>
+      </c>
+      <c r="X2" s="6" t="inlineStr">
         <is>
           <t>Overall Score (1-5)</t>
         </is>
       </c>
-      <c r="X2" s="7" t="inlineStr">
+      <c r="Y2" s="7" t="inlineStr">
         <is>
           <t>Main Element Present?</t>
         </is>
       </c>
-      <c r="Y2" s="7" t="inlineStr">
+      <c r="Z2" s="7" t="inlineStr">
         <is>
           <t>Supporting Element(s) Present?</t>
         </is>
       </c>
-      <c r="Z2" s="7" t="inlineStr">
+      <c r="AA2" s="7" t="inlineStr">
         <is>
           <t>Track Style Visible?</t>
         </is>
       </c>
-      <c r="AA2" s="7" t="inlineStr">
+      <c r="AB2" s="7" t="inlineStr">
         <is>
           <t>Mood / Lighting Correct?</t>
         </is>
       </c>
-      <c r="AB2" s="7" t="inlineStr">
+      <c r="AC2" s="7" t="inlineStr">
         <is>
           <t>Text Zone Clear?</t>
         </is>
       </c>
-      <c r="AC2" s="8" t="inlineStr">
+      <c r="AD2" s="8" t="inlineStr">
         <is>
           <t>Colour Harmony (1-5)</t>
         </is>
       </c>
-      <c r="AD2" s="8" t="inlineStr">
+      <c r="AE2" s="8" t="inlineStr">
         <is>
           <t>WhatsApp-Ready?</t>
         </is>
       </c>
-      <c r="AE2" s="8" t="inlineStr">
+      <c r="AF2" s="8" t="inlineStr">
         <is>
           <t>Failure Tags</t>
         </is>
       </c>
-      <c r="AF2" s="9" t="inlineStr">
+      <c r="AG2" s="9" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
@@ -856,15 +994,16 @@
       <c r="U3" s="11" t="n"/>
       <c r="V3" s="11" t="n"/>
       <c r="W3" s="11" t="n"/>
-      <c r="X3" s="11" t="n"/>
-      <c r="Y3" s="11" t="n"/>
-      <c r="Z3" s="11" t="n"/>
-      <c r="AA3" s="11" t="n"/>
-      <c r="AB3" s="11" t="n"/>
-      <c r="AC3" s="11" t="n"/>
-      <c r="AD3" s="11" t="n"/>
-      <c r="AE3" s="11" t="n"/>
-      <c r="AF3" s="11" t="n"/>
+      <c r="X3" s="10" t="n"/>
+      <c r="Y3" s="10" t="n"/>
+      <c r="Z3" s="10" t="n"/>
+      <c r="AA3" s="10" t="n"/>
+      <c r="AB3" s="10" t="n"/>
+      <c r="AC3" s="10" t="n"/>
+      <c r="AD3" s="10" t="n"/>
+      <c r="AE3" s="10" t="n"/>
+      <c r="AF3" s="10" t="n"/>
+      <c r="AG3" s="10" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="12" t="n"/>
@@ -889,7 +1028,7 @@
       <c r="T4" s="13" t="n"/>
       <c r="U4" s="13" t="n"/>
       <c r="V4" s="13" t="n"/>
-      <c r="W4" s="14" t="n"/>
+      <c r="W4" s="13" t="n"/>
       <c r="X4" s="14" t="n"/>
       <c r="Y4" s="14" t="n"/>
       <c r="Z4" s="14" t="n"/>
@@ -899,6 +1038,7 @@
       <c r="AD4" s="14" t="n"/>
       <c r="AE4" s="14" t="n"/>
       <c r="AF4" s="14" t="n"/>
+      <c r="AG4" s="14" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="10" t="n"/>
@@ -924,15 +1064,16 @@
       <c r="U5" s="11" t="n"/>
       <c r="V5" s="11" t="n"/>
       <c r="W5" s="11" t="n"/>
-      <c r="X5" s="11" t="n"/>
-      <c r="Y5" s="11" t="n"/>
-      <c r="Z5" s="11" t="n"/>
-      <c r="AA5" s="11" t="n"/>
-      <c r="AB5" s="11" t="n"/>
-      <c r="AC5" s="11" t="n"/>
-      <c r="AD5" s="11" t="n"/>
-      <c r="AE5" s="11" t="n"/>
-      <c r="AF5" s="11" t="n"/>
+      <c r="X5" s="10" t="n"/>
+      <c r="Y5" s="10" t="n"/>
+      <c r="Z5" s="10" t="n"/>
+      <c r="AA5" s="10" t="n"/>
+      <c r="AB5" s="10" t="n"/>
+      <c r="AC5" s="10" t="n"/>
+      <c r="AD5" s="10" t="n"/>
+      <c r="AE5" s="10" t="n"/>
+      <c r="AF5" s="10" t="n"/>
+      <c r="AG5" s="10" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="12" t="n"/>
@@ -957,7 +1098,7 @@
       <c r="T6" s="13" t="n"/>
       <c r="U6" s="13" t="n"/>
       <c r="V6" s="13" t="n"/>
-      <c r="W6" s="14" t="n"/>
+      <c r="W6" s="13" t="n"/>
       <c r="X6" s="14" t="n"/>
       <c r="Y6" s="14" t="n"/>
       <c r="Z6" s="14" t="n"/>
@@ -967,6 +1108,7 @@
       <c r="AD6" s="14" t="n"/>
       <c r="AE6" s="14" t="n"/>
       <c r="AF6" s="14" t="n"/>
+      <c r="AG6" s="14" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="10" t="n"/>
@@ -992,15 +1134,16 @@
       <c r="U7" s="11" t="n"/>
       <c r="V7" s="11" t="n"/>
       <c r="W7" s="11" t="n"/>
-      <c r="X7" s="11" t="n"/>
-      <c r="Y7" s="11" t="n"/>
-      <c r="Z7" s="11" t="n"/>
-      <c r="AA7" s="11" t="n"/>
-      <c r="AB7" s="11" t="n"/>
-      <c r="AC7" s="11" t="n"/>
-      <c r="AD7" s="11" t="n"/>
-      <c r="AE7" s="11" t="n"/>
-      <c r="AF7" s="11" t="n"/>
+      <c r="X7" s="10" t="n"/>
+      <c r="Y7" s="10" t="n"/>
+      <c r="Z7" s="10" t="n"/>
+      <c r="AA7" s="10" t="n"/>
+      <c r="AB7" s="10" t="n"/>
+      <c r="AC7" s="10" t="n"/>
+      <c r="AD7" s="10" t="n"/>
+      <c r="AE7" s="10" t="n"/>
+      <c r="AF7" s="10" t="n"/>
+      <c r="AG7" s="10" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="12" t="n"/>
@@ -1025,7 +1168,7 @@
       <c r="T8" s="13" t="n"/>
       <c r="U8" s="13" t="n"/>
       <c r="V8" s="13" t="n"/>
-      <c r="W8" s="14" t="n"/>
+      <c r="W8" s="13" t="n"/>
       <c r="X8" s="14" t="n"/>
       <c r="Y8" s="14" t="n"/>
       <c r="Z8" s="14" t="n"/>
@@ -1035,6 +1178,7 @@
       <c r="AD8" s="14" t="n"/>
       <c r="AE8" s="14" t="n"/>
       <c r="AF8" s="14" t="n"/>
+      <c r="AG8" s="14" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="10" t="n"/>
@@ -1060,15 +1204,16 @@
       <c r="U9" s="11" t="n"/>
       <c r="V9" s="11" t="n"/>
       <c r="W9" s="11" t="n"/>
-      <c r="X9" s="11" t="n"/>
-      <c r="Y9" s="11" t="n"/>
-      <c r="Z9" s="11" t="n"/>
-      <c r="AA9" s="11" t="n"/>
-      <c r="AB9" s="11" t="n"/>
-      <c r="AC9" s="11" t="n"/>
-      <c r="AD9" s="11" t="n"/>
-      <c r="AE9" s="11" t="n"/>
-      <c r="AF9" s="11" t="n"/>
+      <c r="X9" s="10" t="n"/>
+      <c r="Y9" s="10" t="n"/>
+      <c r="Z9" s="10" t="n"/>
+      <c r="AA9" s="10" t="n"/>
+      <c r="AB9" s="10" t="n"/>
+      <c r="AC9" s="10" t="n"/>
+      <c r="AD9" s="10" t="n"/>
+      <c r="AE9" s="10" t="n"/>
+      <c r="AF9" s="10" t="n"/>
+      <c r="AG9" s="10" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="12" t="n"/>
@@ -1093,7 +1238,7 @@
       <c r="T10" s="13" t="n"/>
       <c r="U10" s="13" t="n"/>
       <c r="V10" s="13" t="n"/>
-      <c r="W10" s="14" t="n"/>
+      <c r="W10" s="13" t="n"/>
       <c r="X10" s="14" t="n"/>
       <c r="Y10" s="14" t="n"/>
       <c r="Z10" s="14" t="n"/>
@@ -1103,6 +1248,7 @@
       <c r="AD10" s="14" t="n"/>
       <c r="AE10" s="14" t="n"/>
       <c r="AF10" s="14" t="n"/>
+      <c r="AG10" s="14" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="10" t="n"/>
@@ -1128,42 +1274,43 @@
       <c r="U11" s="11" t="n"/>
       <c r="V11" s="11" t="n"/>
       <c r="W11" s="11" t="n"/>
-      <c r="X11" s="11" t="n"/>
-      <c r="Y11" s="11" t="n"/>
-      <c r="Z11" s="11" t="n"/>
-      <c r="AA11" s="11" t="n"/>
-      <c r="AB11" s="11" t="n"/>
-      <c r="AC11" s="11" t="n"/>
-      <c r="AD11" s="11" t="n"/>
-      <c r="AE11" s="11" t="n"/>
-      <c r="AF11" s="11" t="n"/>
+      <c r="X11" s="10" t="n"/>
+      <c r="Y11" s="10" t="n"/>
+      <c r="Z11" s="10" t="n"/>
+      <c r="AA11" s="10" t="n"/>
+      <c r="AB11" s="10" t="n"/>
+      <c r="AC11" s="10" t="n"/>
+      <c r="AD11" s="10" t="n"/>
+      <c r="AE11" s="10" t="n"/>
+      <c r="AF11" s="10" t="n"/>
+      <c r="AG11" s="10" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="5">
-    <mergeCell ref="AC1:AE1"/>
-    <mergeCell ref="X1:AB1"/>
-    <mergeCell ref="A1:V1"/>
-    <mergeCell ref="AF1"/>
-    <mergeCell ref="W1"/>
+    <mergeCell ref="AD1:AF1"/>
+    <mergeCell ref="A1:W1"/>
+    <mergeCell ref="X1"/>
+    <mergeCell ref="Y1:AC1"/>
+    <mergeCell ref="AG1"/>
   </mergeCells>
   <dataValidations count="7">
-    <dataValidation sqref="W3:W502" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid Score" error="Enter 1-5" promptTitle="Overall Score" prompt="1=Unusable, 2=Poor, 3=Decent, 4=Good, 5=Ship it" type="list">
+    <dataValidation sqref="X3:X502" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid Score" error="Enter 1-5" promptTitle="Overall Score" prompt="1=Unusable, 2=Poor, 3=Decent, 4=Good, 5=Ship it" type="list">
       <formula1>"1,2,3,4,5"</formula1>
     </dataValidation>
-    <dataValidation sqref="X3:X502 Y3:Y502 Z3:Z502 AA3:AA502 AB3:AB502" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid" error="Enter Y, P, or N" promptTitle="Element Check" prompt="Y=Yes, P=Partial, N=No/Missing" type="list">
+    <dataValidation sqref="Y3:Y502 Z3:Z502 AA3:AA502 AB3:AB502 AC3:AC502" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid" error="Enter Y, P, or N" promptTitle="Element Check" prompt="Y=Yes, P=Partial, N=No/Missing" type="list">
       <formula1>"Y,P,N"</formula1>
     </dataValidation>
-    <dataValidation sqref="AC3:AC502" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" promptTitle="Colour Harmony" prompt="1=Clash, 3=Ok, 5=Beautiful" type="list">
+    <dataValidation sqref="AD3:AD502" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" promptTitle="Colour Harmony" prompt="1=Clash, 3=Ok, 5=Beautiful" type="list">
       <formula1>"1,2,3,4,5"</formula1>
     </dataValidation>
-    <dataValidation sqref="AD3:AD502" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" promptTitle="WhatsApp-Ready" prompt="Would a user forward this?" type="list">
+    <dataValidation sqref="AE3:AE502" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" promptTitle="WhatsApp-Ready" prompt="Would a user forward this?" type="list">
       <formula1>"Y,N"</formula1>
     </dataValidation>
-    <dataValidation sqref="AE3:AE502" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" promptTitle="Failure Tag" prompt="Select primary failure (or None)" type="list">
+    <dataValidation sqref="AF3:AF502" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" promptTitle="Failure Tag" prompt="Select primary failure (or None)" type="list">
       <formula1>"Wrong style,Missing element,Bad crop,Artifacts/distortion,Too dark,Too busy,Elements merged,Cartoon leak,Text zone blocked,Colour mismatch,None"</formula1>
     </dataValidation>
     <dataValidation sqref="S3:S502" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" promptTitle="Platform" prompt="Which platform was this run on?" type="list">
-      <formula1>"Midjourney,Leonardo.AI,Adobe Firefly"</formula1>
+      <formula1>"Midjourney,Leonardo.AI,Adobe Firefly,Google Gemini"</formula1>
     </dataValidation>
     <dataValidation sqref="D3:D502" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"A1,A2,B1"</formula1>
@@ -1277,7 +1424,7 @@
     <row r="13">
       <c r="A13" s="18" t="inlineStr">
         <is>
-          <t>PART A — AUTO-FILLED COLUMNS (Cols A–V)</t>
+          <t>PART A — AUTO-FILLED COLUMNS (Cols A–W)</t>
         </is>
       </c>
       <c r="B13" t="inlineStr"/>
@@ -1353,7 +1500,7 @@
     <row r="20">
       <c r="A20" s="16" t="inlineStr">
         <is>
-          <t>Prompts (MJ / Leonardo / Firefly) — full prompt text</t>
+          <t>Prompts (MJ / Leonardo / Firefly / Gemini) — full prompt text</t>
         </is>
       </c>
       <c r="B20" s="17" t="inlineStr">
@@ -1369,7 +1516,7 @@
     <row r="22">
       <c r="A22" s="18" t="inlineStr">
         <is>
-          <t>PART B — HUMAN-RATED COLUMNS (Cols W–AF)</t>
+          <t>PART B — HUMAN-RATED COLUMNS (Cols X–AG)</t>
         </is>
       </c>
       <c r="B22" t="inlineStr"/>
@@ -1509,7 +1656,7 @@
     <row r="35">
       <c r="A35" s="16" t="inlineStr">
         <is>
-          <t>• Paste one row per platform test (same choices, different platform = 3 rows)</t>
+          <t>• Paste one row per platform test (same choices, different platform = 4 rows)</t>
         </is>
       </c>
       <c r="B35" s="17" t="inlineStr"/>
@@ -1549,7 +1696,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G37"/>
+  <dimension ref="A1:G38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -1799,7 +1946,11 @@
       <c r="G17" s="22" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="16" t="inlineStr"/>
+      <c r="A18" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Google Gemini</t>
+        </is>
+      </c>
       <c r="B18" s="22" t="n"/>
       <c r="C18" s="22" t="n"/>
       <c r="D18" s="22" t="n"/>
@@ -1808,11 +1959,7 @@
       <c r="G18" s="22" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="21" t="inlineStr">
-        <is>
-          <t>By Mood (B1)</t>
-        </is>
-      </c>
+      <c r="A19" s="16" t="inlineStr"/>
       <c r="B19" s="22" t="n"/>
       <c r="C19" s="22" t="n"/>
       <c r="D19" s="22" t="n"/>
@@ -1821,9 +1968,9 @@
       <c r="G19" s="22" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Golden Warm</t>
+      <c r="A20" s="21" t="inlineStr">
+        <is>
+          <t>By Mood (B1)</t>
         </is>
       </c>
       <c r="B20" s="22" t="n"/>
@@ -1836,7 +1983,7 @@
     <row r="21">
       <c r="A21" s="16" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Misty Soft</t>
+          <t xml:space="preserve">  Golden Warm</t>
         </is>
       </c>
       <c r="B21" s="22" t="n"/>
@@ -1849,7 +1996,7 @@
     <row r="22">
       <c r="A22" s="16" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Bright &amp; Vivid</t>
+          <t xml:space="preserve">  Misty Soft</t>
         </is>
       </c>
       <c r="B22" s="22" t="n"/>
@@ -1862,7 +2009,7 @@
     <row r="23">
       <c r="A23" s="16" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Dramatic Rays</t>
+          <t xml:space="preserve">  Bright &amp; Vivid</t>
         </is>
       </c>
       <c r="B23" s="22" t="n"/>
@@ -1875,7 +2022,7 @@
     <row r="24">
       <c r="A24" s="16" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Vintage Film</t>
+          <t xml:space="preserve">  Dramatic Rays</t>
         </is>
       </c>
       <c r="B24" s="22" t="n"/>
@@ -1888,7 +2035,7 @@
     <row r="25">
       <c r="A25" s="16" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Soft Pastel</t>
+          <t xml:space="preserve">  Vintage Film</t>
         </is>
       </c>
       <c r="B25" s="22" t="n"/>
@@ -1899,7 +2046,11 @@
       <c r="G25" s="22" t="n"/>
     </row>
     <row r="26">
-      <c r="A26" s="16" t="inlineStr"/>
+      <c r="A26" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Soft Pastel</t>
+        </is>
+      </c>
       <c r="B26" s="22" t="n"/>
       <c r="C26" s="22" t="n"/>
       <c r="D26" s="22" t="n"/>
@@ -1908,11 +2059,7 @@
       <c r="G26" s="22" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" s="21" t="inlineStr">
-        <is>
-          <t>By Overlay</t>
-        </is>
-      </c>
+      <c r="A27" s="16" t="inlineStr"/>
       <c r="B27" s="22" t="n"/>
       <c r="C27" s="22" t="n"/>
       <c r="D27" s="22" t="n"/>
@@ -1921,9 +2068,9 @@
       <c r="G27" s="22" t="n"/>
     </row>
     <row r="28">
-      <c r="A28" s="16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  O1 Full Dark</t>
+      <c r="A28" s="21" t="inlineStr">
+        <is>
+          <t>By Overlay</t>
         </is>
       </c>
       <c r="B28" s="22" t="n"/>
@@ -1936,7 +2083,7 @@
     <row r="29">
       <c r="A29" s="16" t="inlineStr">
         <is>
-          <t xml:space="preserve">  O2 Gradient Top</t>
+          <t xml:space="preserve">  O1 Full Dark</t>
         </is>
       </c>
       <c r="B29" s="22" t="n"/>
@@ -1949,7 +2096,7 @@
     <row r="30">
       <c r="A30" s="16" t="inlineStr">
         <is>
-          <t xml:space="preserve">  O3 Gradient Bottom</t>
+          <t xml:space="preserve">  O2 Gradient Top</t>
         </is>
       </c>
       <c r="B30" s="22" t="n"/>
@@ -1962,7 +2109,7 @@
     <row r="31">
       <c r="A31" s="16" t="inlineStr">
         <is>
-          <t xml:space="preserve">  O4 Vignette</t>
+          <t xml:space="preserve">  O3 Gradient Bottom</t>
         </is>
       </c>
       <c r="B31" s="22" t="n"/>
@@ -1975,7 +2122,7 @@
     <row r="32">
       <c r="A32" s="16" t="inlineStr">
         <is>
-          <t xml:space="preserve">  O5 Caption Bar</t>
+          <t xml:space="preserve">  O4 Vignette</t>
         </is>
       </c>
       <c r="B32" s="22" t="n"/>
@@ -1986,7 +2133,11 @@
       <c r="G32" s="22" t="n"/>
     </row>
     <row r="33">
-      <c r="A33" s="16" t="inlineStr"/>
+      <c r="A33" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  O5 Caption Bar</t>
+        </is>
+      </c>
       <c r="B33" s="22" t="n"/>
       <c r="C33" s="22" t="n"/>
       <c r="D33" s="22" t="n"/>
@@ -1995,11 +2146,7 @@
       <c r="G33" s="22" t="n"/>
     </row>
     <row r="34">
-      <c r="A34" s="21" t="inlineStr">
-        <is>
-          <t>By Intensity</t>
-        </is>
-      </c>
+      <c r="A34" s="16" t="inlineStr"/>
       <c r="B34" s="22" t="n"/>
       <c r="C34" s="22" t="n"/>
       <c r="D34" s="22" t="n"/>
@@ -2008,9 +2155,9 @@
       <c r="G34" s="22" t="n"/>
     </row>
     <row r="35">
-      <c r="A35" s="16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Basic</t>
+      <c r="A35" s="21" t="inlineStr">
+        <is>
+          <t>By Intensity</t>
         </is>
       </c>
       <c r="B35" s="22" t="n"/>
@@ -2023,7 +2170,7 @@
     <row r="36">
       <c r="A36" s="16" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Medium</t>
+          <t xml:space="preserve">  Basic</t>
         </is>
       </c>
       <c r="B36" s="22" t="n"/>
@@ -2036,7 +2183,7 @@
     <row r="37">
       <c r="A37" s="16" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Complex</t>
+          <t xml:space="preserve">  Medium</t>
         </is>
       </c>
       <c r="B37" s="22" t="n"/>
@@ -2046,7 +2193,690 @@
       <c r="F37" s="22" t="n"/>
       <c r="G37" s="22" t="n"/>
     </row>
+    <row r="38">
+      <c r="A38" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Complex</t>
+        </is>
+      </c>
+      <c r="B38" s="22" t="n"/>
+      <c r="C38" s="22" t="n"/>
+      <c r="D38" s="22" t="n"/>
+      <c r="E38" s="22" t="n"/>
+      <c r="F38" s="22" t="n"/>
+      <c r="G38" s="22" t="n"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D46"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="70" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="32" customHeight="1">
+      <c r="A1" s="23" t="inlineStr">
+        <is>
+          <t>QA Testing Guide — What to Check Per Track</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="17" t="inlineStr">
+        <is>
+          <t>Use this checklist while scoring each generated image. Check the items relevant to the Track and Archetype you selected.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="26" customHeight="1">
+      <c r="A4" s="24" t="inlineStr">
+        <is>
+          <t>GENERAL CHECKS (All Tracks)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="32" customHeight="1">
+      <c r="A5" s="25" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B5" s="26" t="inlineStr">
+        <is>
+          <t>Is there a clear text zone (empty area for Good Morning text overlay)?</t>
+        </is>
+      </c>
+      <c r="C5" s="27" t="inlineStr">
+        <is>
+          <t>→ Text Zone Clear?</t>
+        </is>
+      </c>
+      <c r="D5" s="28" t="inlineStr">
+        <is>
+          <t>If text zone is cluttered, mark N. Partial clutter = P.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="32" customHeight="1">
+      <c r="A6" s="25" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B6" s="26" t="inlineStr">
+        <is>
+          <t>Is the main illustration/subject clearly visible and recognisable?</t>
+        </is>
+      </c>
+      <c r="C6" s="27" t="inlineStr">
+        <is>
+          <t>→ Main Element Present?</t>
+        </is>
+      </c>
+      <c r="D6" s="28" t="inlineStr">
+        <is>
+          <t>Distorted or merged with background = P.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="32" customHeight="1">
+      <c r="A7" s="25" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B7" s="26" t="inlineStr">
+        <is>
+          <t>Are supporting elements (motifs, secondary items) present if selected?</t>
+        </is>
+      </c>
+      <c r="C7" s="27" t="inlineStr">
+        <is>
+          <t>→ Supporting Element(s)?</t>
+        </is>
+      </c>
+      <c r="D7" s="28" t="inlineStr">
+        <is>
+          <t>Mark N/A for single-element A1/A2 setups.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="32" customHeight="1">
+      <c r="A8" s="25" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B8" s="26" t="inlineStr">
+        <is>
+          <t>Is the overall composition clean — no weird artifacts, extra limbs, or distortions?</t>
+        </is>
+      </c>
+      <c r="C8" s="27" t="inlineStr">
+        <is>
+          <t>→ Failure Tags</t>
+        </is>
+      </c>
+      <c r="D8" s="28" t="inlineStr">
+        <is>
+          <t>Tag 'Artifacts/distortion' if AI hallucinated extra elements.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="32" customHeight="1">
+      <c r="A9" s="25" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B9" s="26" t="inlineStr">
+        <is>
+          <t>Does the colour palette feel harmonious and intentional?</t>
+        </is>
+      </c>
+      <c r="C9" s="27" t="inlineStr">
+        <is>
+          <t>→ Colour Harmony (1-5)</t>
+        </is>
+      </c>
+      <c r="D9" s="28" t="inlineStr">
+        <is>
+          <t>1=Clashing jarring colours, 3=OK, 5=Beautiful harmony.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="32" customHeight="1">
+      <c r="A10" s="25" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B10" s="26" t="inlineStr">
+        <is>
+          <t>Would you send this on WhatsApp as a Good Morning image?</t>
+        </is>
+      </c>
+      <c r="C10" s="27" t="inlineStr">
+        <is>
+          <t>→ WhatsApp-Ready?</t>
+        </is>
+      </c>
+      <c r="D10" s="28" t="inlineStr">
+        <is>
+          <t>The ultimate test — would a real user forward this?</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="28" customHeight="1">
+      <c r="A12" s="29" t="inlineStr">
+        <is>
+          <t>Track A — Shiny Maximal ✨</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="30" t="inlineStr">
+        <is>
+          <t>Jazzy desi, festive, loud on purpose. Wedding-card meets Diwali poster energy.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="31" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B14" s="32" t="inlineStr">
+        <is>
+          <t>What to Check</t>
+        </is>
+      </c>
+      <c r="C14" s="32" t="inlineStr">
+        <is>
+          <t>Maps to Column</t>
+        </is>
+      </c>
+      <c r="D14" s="32" t="inlineStr">
+        <is>
+          <t>Scoring Tip</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="36" customHeight="1">
+      <c r="A15" s="33" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B15" s="34" t="inlineStr">
+        <is>
+          <t>WATCH OUT: Should NOT look minimalist, muted, earthy, or grayscale</t>
+        </is>
+      </c>
+      <c r="C15" s="35" t="inlineStr">
+        <is>
+          <t>→ Failure Tags</t>
+        </is>
+      </c>
+      <c r="D15" s="36" t="inlineStr">
+        <is>
+          <t>Tag 'Wrong style' if it looks like Track B/C/E instead.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="28" customHeight="1">
+      <c r="A17" s="37" t="inlineStr">
+        <is>
+          <t>Track B — Modern Desi 🎨</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="30" t="inlineStr">
+        <is>
+          <t>Muted earthy, contemporary editorial. Restrained Indian design.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="31" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B19" s="32" t="inlineStr">
+        <is>
+          <t>What to Check</t>
+        </is>
+      </c>
+      <c r="C19" s="32" t="inlineStr">
+        <is>
+          <t>Maps to Column</t>
+        </is>
+      </c>
+      <c r="D19" s="32" t="inlineStr">
+        <is>
+          <t>Scoring Tip</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="36" customHeight="1">
+      <c r="A20" s="33" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B20" s="34" t="inlineStr">
+        <is>
+          <t>WATCH OUT: Should NOT have gold foil, sparkle, metallic, or loud vivid colours</t>
+        </is>
+      </c>
+      <c r="C20" s="35" t="inlineStr">
+        <is>
+          <t>→ Failure Tags</t>
+        </is>
+      </c>
+      <c r="D20" s="36" t="inlineStr">
+        <is>
+          <t>Tag 'Wrong style' if it looks like Track A.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="28" customHeight="1">
+      <c r="A22" s="38" t="inlineStr">
+        <is>
+          <t>Track C — Minimalist Classy 🎬</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="30" t="inlineStr">
+        <is>
+          <t>Maximum restraint, tonal elegance, single focal element. Premium minimal.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="31" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B24" s="32" t="inlineStr">
+        <is>
+          <t>What to Check</t>
+        </is>
+      </c>
+      <c r="C24" s="32" t="inlineStr">
+        <is>
+          <t>Maps to Column</t>
+        </is>
+      </c>
+      <c r="D24" s="32" t="inlineStr">
+        <is>
+          <t>Scoring Tip</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="36" customHeight="1">
+      <c r="A25" s="33" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B25" s="34" t="inlineStr">
+        <is>
+          <t>WATCH OUT: Should NOT have gradients, ornate borders, gold foil, busy patterns, or doodles</t>
+        </is>
+      </c>
+      <c r="C25" s="35" t="inlineStr">
+        <is>
+          <t>→ Failure Tags</t>
+        </is>
+      </c>
+      <c r="D25" s="36" t="inlineStr">
+        <is>
+          <t>Tag 'Wrong style' if it feels busy, festive, or handmade.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="28" customHeight="1">
+      <c r="A27" s="39" t="inlineStr">
+        <is>
+          <t>Track D — Artsy Playful 🎉</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="30" t="inlineStr">
+        <is>
+          <t>Flat bright, sticker/doodle aesthetic, cheerful Gen-Z energy.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="31" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B29" s="32" t="inlineStr">
+        <is>
+          <t>What to Check</t>
+        </is>
+      </c>
+      <c r="C29" s="32" t="inlineStr">
+        <is>
+          <t>Maps to Column</t>
+        </is>
+      </c>
+      <c r="D29" s="32" t="inlineStr">
+        <is>
+          <t>Scoring Tip</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="36" customHeight="1">
+      <c r="A30" s="33" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B30" s="34" t="inlineStr">
+        <is>
+          <t>WATCH OUT: Should NOT look photorealistic, ornate, gold, muted, or serif-heavy</t>
+        </is>
+      </c>
+      <c r="C30" s="35" t="inlineStr">
+        <is>
+          <t>→ Failure Tags</t>
+        </is>
+      </c>
+      <c r="D30" s="36" t="inlineStr">
+        <is>
+          <t>Tag 'Wrong style' if it feels like Track A (ornate) or Track C (minimal).</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="28" customHeight="1">
+      <c r="A32" s="40" t="inlineStr">
+        <is>
+          <t>Track E — Soft &amp; Warm 🌷</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="30" t="inlineStr">
+        <is>
+          <t>Gentle pastels, warm botanicals, calming morning energy. Soft and feminine.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="31" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B34" s="32" t="inlineStr">
+        <is>
+          <t>What to Check</t>
+        </is>
+      </c>
+      <c r="C34" s="32" t="inlineStr">
+        <is>
+          <t>Maps to Column</t>
+        </is>
+      </c>
+      <c r="D34" s="32" t="inlineStr">
+        <is>
+          <t>Scoring Tip</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="36" customHeight="1">
+      <c r="A35" s="33" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B35" s="34" t="inlineStr">
+        <is>
+          <t>WATCH OUT: Should NOT have neon, metallic, glitter, bold outlines, or sharp vector edges</t>
+        </is>
+      </c>
+      <c r="C35" s="35" t="inlineStr">
+        <is>
+          <t>→ Failure Tags</t>
+        </is>
+      </c>
+      <c r="D35" s="36" t="inlineStr">
+        <is>
+          <t>Tag 'Wrong style' if it feels bold, flashy, or sharp-edged.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="28" customHeight="1">
+      <c r="A37" s="41" t="inlineStr">
+        <is>
+          <t>B1 — Photo Background Specific Checks</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="30" t="inlineStr">
+        <is>
+          <t>These apply to ALL B1 outputs regardless of track. Check these IN ADDITION to the track checks above.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="42" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B39" s="42" t="inlineStr">
+        <is>
+          <t>What to Check</t>
+        </is>
+      </c>
+      <c r="C39" s="42" t="inlineStr">
+        <is>
+          <t>Maps to Column</t>
+        </is>
+      </c>
+      <c r="D39" s="42" t="inlineStr">
+        <is>
+          <t>Scoring Tip</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="30" customHeight="1">
+      <c r="A40" s="43" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B40" s="44" t="inlineStr">
+        <is>
+          <t>Is it a real photograph — not an illustration, painting, or cartoon?</t>
+        </is>
+      </c>
+      <c r="C40" s="45" t="inlineStr">
+        <is>
+          <t>→ Track Style Visible?</t>
+        </is>
+      </c>
+      <c r="D40" s="46" t="inlineStr">
+        <is>
+          <t>B1 = photorealistic only. Any cartoon/vector leak = tag 'Cartoon leak'.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="30" customHeight="1">
+      <c r="A41" s="43" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B41" s="44" t="inlineStr">
+        <is>
+          <t>Is the image truly full-bleed (no frame, no border, edge-to-edge photo)?</t>
+        </is>
+      </c>
+      <c r="C41" s="45" t="inlineStr">
+        <is>
+          <t>→ Main Element Present?</t>
+        </is>
+      </c>
+      <c r="D41" s="46" t="inlineStr">
+        <is>
+          <t>Frames/borders are A1/A2 only. B1 must be frameless.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="30" customHeight="1">
+      <c r="A42" s="43" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B42" s="44" t="inlineStr">
+        <is>
+          <t>Does the mood/lighting match the selection? (golden warm, misty, dramatic, etc.)</t>
+        </is>
+      </c>
+      <c r="C42" s="45" t="inlineStr">
+        <is>
+          <t>→ Mood / Lighting?</t>
+        </is>
+      </c>
+      <c r="D42" s="46" t="inlineStr">
+        <is>
+          <t>Compare against the mood you selected in the wizard.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="30" customHeight="1">
+      <c r="A43" s="43" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B43" s="44" t="inlineStr">
+        <is>
+          <t>Is the overlay correct? (dark gradient at bottom, vignette, caption bar, etc.)</t>
+        </is>
+      </c>
+      <c r="C43" s="45" t="inlineStr">
+        <is>
+          <t>→ Mood / Lighting?</t>
+        </is>
+      </c>
+      <c r="D43" s="46" t="inlineStr">
+        <is>
+          <t>The overlay creates the text-readable zone. Wrong placement = fail.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="30" customHeight="1">
+      <c r="A44" s="43" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B44" s="44" t="inlineStr">
+        <is>
+          <t>Are the main scene elements present? (chai cup, flowers, sunrise, etc.)</t>
+        </is>
+      </c>
+      <c r="C44" s="45" t="inlineStr">
+        <is>
+          <t>→ Main Element Present?</t>
+        </is>
+      </c>
+      <c r="D44" s="46" t="inlineStr">
+        <is>
+          <t>AI sometimes swaps or drops scene elements entirely.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="30" customHeight="1">
+      <c r="A45" s="43" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B45" s="44" t="inlineStr">
+        <is>
+          <t>Does the photo feel like the right photography style for the track?</t>
+        </is>
+      </c>
+      <c r="C45" s="45" t="inlineStr">
+        <is>
+          <t>→ Track Style Visible?</t>
+        </is>
+      </c>
+      <c r="D45" s="46" t="inlineStr">
+        <is>
+          <t>E.g., Track A/B1 = warm saturated, Track C/B1 = clean editorial.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="36" customHeight="1">
+      <c r="A46" s="33" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="B46" s="34" t="inlineStr">
+        <is>
+          <t>WATCH OUT: Any illustration elements, cartoon styling, vector shapes, or painted look = FAIL for B1</t>
+        </is>
+      </c>
+      <c r="C46" s="35" t="inlineStr">
+        <is>
+          <t>→ Failure Tags</t>
+        </is>
+      </c>
+      <c r="D46" s="36" t="inlineStr">
+        <is>
+          <t>Tag 'Cartoon leak' — this is B1's #1 failure mode.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="15">
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A17:D17"/>
+    <mergeCell ref="A18:D18"/>
+    <mergeCell ref="A23:D23"/>
+    <mergeCell ref="A27:D27"/>
+    <mergeCell ref="A37:D37"/>
+    <mergeCell ref="A22:D22"/>
+    <mergeCell ref="A12:D12"/>
+    <mergeCell ref="A4:D4"/>
+    <mergeCell ref="A38:D38"/>
+    <mergeCell ref="A2:D2"/>
+    <mergeCell ref="A33:D33"/>
+    <mergeCell ref="A28:D28"/>
+    <mergeCell ref="A32:D32"/>
+    <mergeCell ref="A13:D13"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>